<commit_message>
Datenstruktur angepasst; Textprovenienz ergänzt
</commit_message>
<xml_diff>
--- a/raw/Werke.xlsx
+++ b/raw/Werke.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikil\Dropbox\Werkdatenbank\Lasso\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikil\IdeaProjects\lassoDBData\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58C8B122-88AE-4ABA-BC52-F78C3B623017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ADAB781-D5F6-4406-84C2-F622DEF7C695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10340" uniqueCount="5571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10339" uniqueCount="5571">
   <si>
     <t>LV</t>
   </si>
@@ -41814,9 +41814,7 @@
       <c r="D1296" s="2" t="s">
         <v>3500</v>
       </c>
-      <c r="E1296" s="2" t="s">
-        <v>3501</v>
-      </c>
+      <c r="E1296" s="2"/>
       <c r="F1296" s="2" t="s">
         <v>3501</v>
       </c>

</xml_diff>

<commit_message>
- Excel Tabelle mit Werkdaten um neue Spalten "Gattung" und "Sprache" erweitert. Datenschema entsprechend angepasst.
</commit_message>
<xml_diff>
--- a/raw/Werke.xlsx
+++ b/raw/Werke.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikil\IdeaProjects\lassoDBData\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7BAE2CB-9370-42E0-BA3B-72C367B2241E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60475F40-7F20-4EBC-8E99-0EA080E1B6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17253,7 +17253,7 @@
         <v>5571</v>
       </c>
       <c r="J5" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -20475,7 +20475,7 @@
         <v>386</v>
       </c>
       <c r="I131" s="2" t="s">
-        <v>5572</v>
+        <v>5571</v>
       </c>
       <c r="J131" t="s">
         <v>16</v>
@@ -20500,7 +20500,7 @@
         <v>389</v>
       </c>
       <c r="I132" s="2" t="s">
-        <v>5572</v>
+        <v>5571</v>
       </c>
       <c r="J132" t="s">
         <v>16</v>
@@ -20527,7 +20527,7 @@
         <v>393</v>
       </c>
       <c r="I133" s="2" t="s">
-        <v>5572</v>
+        <v>5571</v>
       </c>
       <c r="J133" t="s">
         <v>16</v>
@@ -20552,7 +20552,7 @@
         <v>396</v>
       </c>
       <c r="I134" s="2" t="s">
-        <v>5572</v>
+        <v>5571</v>
       </c>
       <c r="J134" t="s">
         <v>16</v>
@@ -20681,7 +20681,7 @@
         <v>413</v>
       </c>
       <c r="I139" s="2" t="s">
-        <v>5572</v>
+        <v>5573</v>
       </c>
       <c r="J139" t="s">
         <v>25</v>
@@ -20706,7 +20706,7 @@
         <v>413</v>
       </c>
       <c r="I140" s="2" t="s">
-        <v>5572</v>
+        <v>5573</v>
       </c>
       <c r="J140" t="s">
         <v>25</v>

</xml_diff>

<commit_message>
Anpassung und Vereinfachung des Datenschemas + Korrektur von Fehlern in den Daten
</commit_message>
<xml_diff>
--- a/raw/Werke.xlsx
+++ b/raw/Werke.xlsx
@@ -12592,11 +12592,14 @@
       </c>
       <c r="E245" s="2" t="inlineStr">
         <is>
-          <t>Anfang von Psalmus 130, Nachdichtung von 
-Clement Marot</t>
-        </is>
-      </c>
-      <c r="F245" s="2" t="n"/>
+          <t>Clément Marot</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>nach Psalmus 130 (Anfang)</t>
+        </is>
+      </c>
       <c r="G245" s="2" t="inlineStr">
         <is>
           <t>GA 2 XVI,IV 1</t>
@@ -35176,7 +35179,7 @@
     <row r="709">
       <c r="A709" s="4" t="inlineStr">
         <is>
-          <t>419-4</t>
+          <t>419-2</t>
         </is>
       </c>
       <c r="B709" s="2" t="inlineStr">
@@ -50831,7 +50834,7 @@
           <t>1576-5</t>
         </is>
       </c>
-      <c r="E1067" t="inlineStr">
+      <c r="F1067" t="inlineStr">
         <is>
           <t>Tischgebet</t>
         </is>
@@ -50879,7 +50882,7 @@
           <t>1576-7</t>
         </is>
       </c>
-      <c r="E1068" t="inlineStr">
+      <c r="F1068" t="inlineStr">
         <is>
           <t>Tischgebet</t>
         </is>
@@ -86414,12 +86417,12 @@
           <t>1597-1</t>
         </is>
       </c>
-      <c r="E1841" s="2" t="inlineStr">
+      <c r="E1841" s="2" t="n"/>
+      <c r="F1841" s="2" t="inlineStr">
         <is>
           <t>Gebet?</t>
         </is>
       </c>
-      <c r="F1841" s="2" t="n"/>
       <c r="G1841" s="2" t="inlineStr">
         <is>
           <t>GA IX 289</t>
@@ -86578,12 +86581,12 @@
           <t>1597-1</t>
         </is>
       </c>
-      <c r="E1844" s="2" t="inlineStr">
+      <c r="E1844" s="2" t="n"/>
+      <c r="F1844" s="2" t="inlineStr">
         <is>
           <t>Schäfergedicht</t>
         </is>
       </c>
-      <c r="F1844" s="2" t="n"/>
       <c r="G1844" s="2" t="inlineStr">
         <is>
           <t>GA XI 302</t>
@@ -88298,12 +88301,12 @@
           <t>1604-1</t>
         </is>
       </c>
-      <c r="E1882" s="2" t="inlineStr">
+      <c r="E1882" s="2" t="n"/>
+      <c r="F1882" s="2" t="inlineStr">
         <is>
           <t>Tischgebet</t>
         </is>
       </c>
-      <c r="F1882" s="2" t="n"/>
       <c r="G1882" s="2" t="inlineStr">
         <is>
           <t>GA I 46</t>

</xml_diff>